<commit_message>
Finalise submission: P01/P08 rulings, RAM measurement, PDF report, group members
- P01 ruled from the official circular (no attendance requirement to sit the
  Major exam); P08 kept (19-26 Nov 2026). Answers re-scored, no model re-run:
  Qwen3 multi 79%, single 58%, Llama 3.1 multi 50%.
- Add eval/check_sources.py (reference key facts vs cited pages) and
  eval/measure_ram.ps1 (peak RAM: ~6.2 GB for the stack on a 15.7 GB laptop).
- Build REPORT.pdf from REPORT.md (scripts/build_report_pdf.py); add group
  members to the report.
- Rewrite README as a final submission document (remove hand-over/to-do parts).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval/review/question_answer_sheet.xlsx
+++ b/eval/review/question_answer_sheet.xlsx
@@ -728,19 +728,19 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Revised policy (Circular 08-07-2024): "students' examination performance is no longer linked to their course attendance ... In any case, the attendance of a student should not fall below 75% in a course."
+          <t>There is no attendance requirement to sit the Major exam. Circular 08-07-2024: "students' examination performance is no longer linked to their course attendance"; the student is still expected to have full attendance and "in any case, the attendance of a student should not fall below 75% in a course" (below 75% without a valid reason, the instructor can recommend de-registration from the course).
 NOTE: PLEASE JUDGE: the circular says attendance 'should not fall below 75%' but ALSO that exam performance is 'no longer linked to attendance' and students may still appear. Strictly, there may be NO attendance requirement to sit the exam. The scorer only checks that '75%' is mentioned, so an answer saying 'you need 75% to sit the exam' passes. Should the reference answer say this explicitly?
-(Author's note: Assignment example. D01 p.7 states the superseded policy (below 75% must score at least C); an answer presenting that as current is inaccurate.)</t>
+(Author's note: Assignment example. Ruling (2026-10-30, taking the official circular as true): the revised policy delinks exam performance from attendance and supersedes the earlier policy "in totality", so an answer that makes 75% a condition for sitting the exam, or presents the old rule (below 75% must score at least C) as current, is wrong.)</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>no longer linked or not linked or not dependent or independent of</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>[D08, p.1] (scanned page, text recognised by OCR) … sons, the student has to attend every lecture, tutorial, or lab session. The attendance records must be made available to the student after every lecture. Even if the student's attendance falls below 75%, the student will be allowed to appear for the exams. Students not meeting the attendance criterion of 75% will be required to score at least a C grade to pass a course. These students would be awarded an F grade if their marks are lower than the cut-off for a C grade in a course. Revised Policy: According to the recent Senate  …</t>
+          <t>[D08, p.1] (scanned page, text recognised by OCR) …  awarded an F grade if their marks are lower than the cut-off for a C grade in a course. Revised Policy: According to the recent Senate and Board-approved policy, students' examination performance is no longer linked to their course attendance. As per the amendment in attendance policy a student is expected to have full attendance in each course unless the student takes a leave of absence for valid medical or bonafide reasons. In any case, the attendance of a student should not fall below 75% in a course. The attendance records must be made …</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -1075,7 +1075,8 @@
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>MAJOR Examination, Semester I (2026-27): "19-26 November 2026, Thu- Thu"
-NOTE: PLEASE CHECK: the calendar row is labelled 'MAJOR Examination (Fractal 3 and M.Tech. working professional)'. Do these dates apply to the Major exam of ALL Semester I courses, or only to those groups?</t>
+NOTE: PLEASE CHECK: the calendar row is labelled 'MAJOR Examination (Fractal 3 and M.Tech. working professional)'. Do these dates apply to the Major exam of ALL Semester I courses, or only to those groups?
+(Author's note: Ruling (2026-10-30, taking the official calendar as true): page 2 labels the row "MAJOR Examination (Fractal 3 and M.Tech. working professional)", but the detailed schedule (page 8, row 79) lists "Major Semester Examination, 19-26 Nov 2026" for Semester I without that qualifier, so the dates apply to Semester I.)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -1085,17 +1086,20 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>[D11, p.2] … 2026- 27) 09 August 2027, Mon Minor Examination 15-20 September 2026, Tue- Sun 16-21 February 2027, Tue- Sun 04-06 June 2027, Fri-Sun MAJOR Examination (Fractal 3 and M.Tech. working professional) 19-26 November 2026, Thu- Thu 22-29 April 2027, Thu-Thu 10-13 July 2027, Sat-Tue Last date of submission of online grades 30 November 2026, Mon 3 May 2027, Mon 19 July 2027, Mon Moderation Committee Meeting 1 December 2026, Tue 5 May 2027, Wed 20 July 2027, Tue Last Date for display of Grades for Courses, Projects and Thesis; Last date of submissi …</t>
+          <t>[D11, p.2] … 2026- 27) 09 August 2027, Mon Minor Examination 15-20 September 2026, Tue- Sun 16-21 February 2027, Tue- Sun 04-06 June 2027, Fri-Sun MAJOR Examination (Fractal 3 and M.Tech. working professional) 19-26 November 2026, Thu- Thu 22-29 April 2027, Thu-Thu 10-13 July 2027, Sat-Tue Last date of submission of online grades 30 November 2026, Mon 3 May 2027, Mon 19 July 2027, Mon Moderation Committee Meeting 1 December 2026, Tue 5 May 2027, Wed 20 July 2027, Tue Last Date for display of Grades for Courses, Projects and Thesis; Last date of submissi …
+[D11, p.8] …  Display of all Marks for pre major evaluation components 17 Nov 2026, Tue 20 Apr 2027, Tue 09 July 2027, Fri 78. World Creativity &amp; Innovation Day NA 21 Apr 2027, Wed 79. Major Semester Examination 19-26 Nov 2026, Thu- Thu 22-29 April 2027, Thu- Thu 10-13 July 2027, Sat-Tue 80. Constitution Day 26 Nov 2026, Thu NA 81. Last date of submission of online grades 30 Nov 2026, Mon 3 May 2027, Mon 19 July 2027, Mon 82. Moderation Committee Meeting 1 Dec 2026, Tue 5 May 2027, Wed 20 July 2027, Tue 83. Winter/ Summer Break 2 - 30 Dec …</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>D11: Academic Calendar AY 2026-27, p.2</t>
+          <t>D11: Academic Calendar AY 2026-27, p.2
+D11: Academic Calendar AY 2026-27, p.8</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>data/raw/D11.pdf → PDF page 2</t>
+          <t>data/raw/D11.pdf → PDF page 2
+data/raw/D11.pdf → PDF page 8</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -2571,7 +2575,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr">
@@ -2581,7 +2585,7 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>States 75% but presents the superseded rule (below 75% must score at least a C grade) as current; the 08-07-2024 circular (D08) delinks examination performance from attendance.</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L2" s="8" t="n"/>
@@ -2631,17 +2635,17 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>correct</t>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>wrong</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>auto grade confirmed on review</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L3" s="8" t="n"/>
@@ -2690,17 +2694,17 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>correct</t>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>wrong</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>auto grade confirmed on review</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L4" s="8" t="n"/>
@@ -2749,7 +2753,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
@@ -2759,7 +2763,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>States 75% but presents the superseded rule (below 75% must score at least a C grade) as current; the 08-07-2024 circular (D08) delinks examination performance from attendance.</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L5" s="8" t="n"/>
@@ -2808,17 +2812,17 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>correct</t>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>wrong</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>auto grade confirmed on review</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L6" s="8" t="n"/>
@@ -2867,7 +2871,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -2877,7 +2881,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>States 75% but presents the superseded rule (below 75% must score at least a C grade) as current; the 08-07-2024 circular (D08) delinks examination performance from attendance.</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L7" s="8" t="n"/>
@@ -2926,7 +2930,7 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -2936,7 +2940,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>States 75% but presents the superseded rule (below 75% must score at least a C grade) as current; the 08-07-2024 circular (D08) delinks examination performance from attendance.</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L8" s="8" t="n"/>
@@ -2987,7 +2991,7 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
@@ -2997,7 +3001,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>States 75% but presents the superseded rule (below 75% must score at least a C grade) as current; the 08-07-2024 circular (D08) delinks examination performance from attendance.</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L9" s="8" t="n"/>
@@ -3048,7 +3052,7 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
@@ -3058,7 +3062,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>States 75% but presents the superseded rule (below 75% must score at least a C grade) as current; the 08-07-2024 circular (D08) delinks examination performance from attendance.</t>
+          <t>Makes 75% a condition for sitting the exam and/or presents the superseded C-grade rule as current; the 08-07-2024 circular (D08) says exam performance is no longer linked to attendance (reference ruled 2026-10-30 from the official text).</t>
         </is>
       </c>
       <c r="L10" s="8" t="n"/>

</xml_diff>